<commit_message>
Fix inconsistencies in Excel guide and add missing Power Query exercise
- Align terminology between the guide text and the actual workbook
  columns/sheet names (product type vs. policy type, policies vs.
  claims, agent code naming).
- Add the 08_Power_Query practice sheet that chapter 8 referenced but
  never existed in the workbook.
- Replace the confusing "overall check" formula example in chapter 7
  with a clearer OR-based gate formula that matches the workbook's
  actual solution.
</commit_message>
<xml_diff>
--- a/docs/excel-learning-guide/practice_workbook.xlsx
+++ b/docs/excel-learning-guide/practice_workbook.xlsx
@@ -15,7 +15,8 @@
     <sheet name="05_PivotTable" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="06_Conditional_Formatting" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="07_Data_Quality" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="פתרונות" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="08_Power_Query" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="פתרונות" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -121,6 +122,9 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -489,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -602,21 +606,350 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
+          <t>08_Power_Query — תרגול מודרך (אופציונלי) לניקוי נתונים דרך Power Query</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>פתרונות — נוסחאות פתרון עם הסבר</t>
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>בהצלחה!</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>פתרונות — נסו לבד לפני שאתם מציצים כאן</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>פרק</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>משימה</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>נוסחת פתרון / הסבר</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>מחיר אחרי הנחה</t>
+        </is>
+      </c>
+      <c r="C4" s="13">
+        <f>B4*(1-$H$2)  — ה-$ נועל את H2 כדי שהגרירה לא תזיז אותו</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>סה"כ פרמיה</t>
+        </is>
+      </c>
+      <c r="C5" s="13">
+        <f>SUM(D4:D43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>ממוצע פרמיה</t>
+        </is>
+      </c>
+      <c r="C6" s="13">
+        <f>AVERAGE(D4:D43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>מזהה לקוח חסר</t>
+        </is>
+      </c>
+      <c r="C7" s="13">
+        <f>COUNTBLANK(F4:F43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>כמות P-CAR</t>
+        </is>
+      </c>
+      <c r="C8" s="13">
+        <f>COUNTIF(C4:C43,"P-CAR")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>02</t>
+        </is>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>סה"כ פרמיה ל-P-HEALTH</t>
+        </is>
+      </c>
+      <c r="C9" s="13">
+        <f>SUMIF(C4:C43,"P-HEALTH",D4:D43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>שם סוכן נקי</t>
+        </is>
+      </c>
+      <c r="C10" s="13">
+        <f>PROPER(TRIM(B4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>03</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>כפילות</t>
+        </is>
+      </c>
+      <c r="C11" s="13">
+        <f>IF(COUNTIF($A$4:$A$43,A4)&gt;1,"כפול","ייחודי")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>שם מוצר לפי קוד</t>
+        </is>
+      </c>
+      <c r="C12" s="13">
+        <f>IFERROR(VLOOKUP(B4,$H$5:$I$9,2,FALSE),"קוד לא קיים")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>04</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>שם סוכן לפי קוד</t>
+        </is>
+      </c>
+      <c r="C13" s="13">
+        <f>IFERROR(INDEX($L$5:$L$9,MATCH(D4,$K$5:$K$9,0)),"קוד לא קיים")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>PivotTable</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Insert &gt; PivotTable, Rows=שם סוכן, Values=Sum(פרמיה), Columns=סוג מוצר</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>פרמיה שלילית</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>New Rule &gt; Formula: =$D4&lt;0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>תאריך עתידי</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>New Rule &gt; Formula: =$E4&gt;TODAY()</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>06</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>פוליסה כפולה</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>New Rule &gt; Formula: =COUNTIF($A$4:$A$43,$A4)&gt;1</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr"/>
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>שדה חובה</t>
+        </is>
+      </c>
+      <c r="C18" s="13">
+        <f>IF(F4="","חסר","תקין")</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>בהצלחה!</t>
-        </is>
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>כפילות</t>
+        </is>
+      </c>
+      <c r="C19" s="13">
+        <f>IF(COUNTIF($A$4:$A$43,A4)&gt;1,"כפול","ייחודי")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="inlineStr">
+        <is>
+          <t>החלטה סופית</t>
+        </is>
+      </c>
+      <c r="C20" s="13">
+        <f>IF(OR(G4="חסר",H4="כפול",D4&lt;0,E4&gt;TODAY()),"נדחה","קביל")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7718,318 +8051,109 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>פתרונות — נסו לבד לפני שאתם מציצים כאן</t>
-        </is>
-      </c>
+          <t>פרק 8 — תרגול מודרך: Power Query (אופציונלי, לרמה מתקדמת יותר)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>פרק</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>משימה</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>נוסחת פתרון / הסבר</t>
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>המטרה: לבצע את אותו ניקוי נתונים שעשיתם עם נוסחאות בגיליון '03_ניקוי_נתונים', הפעם דרך Power Query — כלי ה-ETL המובנה של Excel.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>מחיר אחרי הנחה</t>
-        </is>
-      </c>
-      <c r="C4" s="12">
-        <f>B4*(1-$H$2)  — ה-$ נועל את H2 כדי שהגרירה לא תזיז אותו</f>
-        <v/>
-      </c>
+      <c r="A4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>סה"כ פרמיה</t>
-        </is>
-      </c>
-      <c r="C5" s="12">
-        <f>SUM(D4:D43)</f>
-        <v/>
+          <t>שלבים:</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>ממוצע פרמיה</t>
-        </is>
-      </c>
-      <c r="C6" s="12">
-        <f>AVERAGE(D4:D43)</f>
-        <v/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>1. עברו לגיליון '03_ניקוי_נתונים' וסמנו את טווח הנתונים כולל כותרות (A3:D43).</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>מזהה לקוח חסר</t>
-        </is>
-      </c>
-      <c r="C7" s="12">
-        <f>COUNTBLANK(F4:F43)</f>
-        <v/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>2. Data → From Table/Range (אם Excel מבקש, אשרו 'My table has headers').</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>כמות P-CAR</t>
-        </is>
-      </c>
-      <c r="C8" s="12">
-        <f>COUNTIF(C4:C43,"P-CAR")</f>
-        <v/>
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>3. ייפתח חלון Power Query Editor עם עורך שלבים (Applied Steps) בצד.</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>02</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>סה"כ פרמיה ל-P-HEALTH</t>
-        </is>
-      </c>
-      <c r="C9" s="12">
-        <f>SUMIF(C4:C43,"P-HEALTH",D4:D43)</f>
-        <v/>
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>4. סמנו את עמודת 'שם סוכן (מקור - מלוכלך)' ← Transform → Format → Trim, ואז שוב Format → Capitalize Each Word (מקביל ל-TRIM ו-PROPER שעשיתם בנוסחה).</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>שם סוכן נקי</t>
-        </is>
-      </c>
-      <c r="C10" s="12">
-        <f>PROPER(TRIM(B4))</f>
-        <v/>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>5. סמנו את עמודת 'מספר פוליסה (מקור)' ← לחצן ימני ← Remove Duplicates (מקביל לבדיקת הכפילות שעשיתם עם COUNTIF).</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>03</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>כפילות</t>
-        </is>
-      </c>
-      <c r="C11" s="12">
-        <f>IF(COUNTIF($A$4:$A$43,A4)&gt;1,"כפול","ייחודי")</f>
-        <v/>
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>6. שנו את סוג הנתונים (Data Type) של כל עמודה בעזרת הסמל בראש העמודה, כדי לוודא שהפרמיה מזוהה כ-Decimal Number.</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>שם מוצר לפי קוד</t>
-        </is>
-      </c>
-      <c r="C12" s="12">
-        <f>IFERROR(VLOOKUP(B4,$H$5:$I$9,2,FALSE),"קוד לא קיים")</f>
-        <v/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>7. Home → Close &amp; Load — הנתונים הנקיים ייטענו כטבלה חדשה בגיליון חדש.</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>04</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>שם סוכן לפי קוד</t>
-        </is>
-      </c>
-      <c r="C13" s="12">
-        <f>IFERROR(INDEX($L$5:$L$9,MATCH(D4,$K$5:$K$9,0)),"קוד לא קיים")</f>
-        <v/>
-      </c>
+      <c r="A13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>05</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>PivotTable</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>Insert &gt; PivotTable, Rows=שם סוכן, Values=Sum(פרמיה), Columns=סוג מוצר</t>
+          <t>היתרון על פני נוסחאות: כל שלב נשמר ורשום ב-Applied Steps. אם מגיע קובץ חדש עם אותו מבנה, מספיק ללחוץ Data → Refresh All וכל תהליך הניקוי רץ מחדש אוטומטית — בלי לגרור נוסחאות מחדש.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>פרמיה שלילית</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>New Rule &gt; Formula: =$D4&lt;0</t>
-        </is>
-      </c>
+      <c r="A15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
         <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>תאריך עתידי</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>New Rule &gt; Formula: =$E4&gt;TODAY()</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>06</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>פוליסה כפולה</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>New Rule &gt; Formula: =COUNTIF($A$4:$A$43,$A4)&gt;1</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>שדה חובה</t>
-        </is>
-      </c>
-      <c r="C18" s="12">
-        <f>IF(F4="","חסר","תקין")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>כפילות</t>
-        </is>
-      </c>
-      <c r="C19" s="12">
-        <f>IF(COUNTIF($A$4:$A$43,A4)&gt;1,"כפול","ייחודי")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>07</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>החלטה סופית</t>
-        </is>
-      </c>
-      <c r="C20" s="12">
-        <f>IF(OR(G4="חסר",H4="כפול",D4&lt;0,E4&gt;TODAY()),"נדחה","קביל")</f>
-        <v/>
+          <t>לחיזוק: נסו למזג (Merge Queries) את הנתונים הנקיים מול טבלת המוצרים בגיליון '04_VLOOKUP' (עמודות H:I) — זו הדרך של Power Query לעשות VLOOKUP, רק שקופה וניתנת לתיעוד.</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Polish Excel guide: add cheat sheet, glossary, and Data Validation exercise
Local-only commit, not pushed — this content is being migrated to a
dedicated repository per request, so the clinical-dataset-etl remote
branch is intentionally left as-is for now.
</commit_message>
<xml_diff>
--- a/docs/excel-learning-guide/practice_workbook.xlsx
+++ b/docs/excel-learning-guide/practice_workbook.xlsx
@@ -55,7 +55,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +72,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1F8"/>
+        <bgColor rgb="00EAF1F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -101,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -119,9 +125,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
@@ -671,277 +679,277 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>01</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>מחיר אחרי הנחה</t>
         </is>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="15">
         <f>B4*(1-$H$2)  — ה-$ נועל את H2 כדי שהגרירה לא תזיז אותו</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>סה"כ פרמיה</t>
         </is>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="15">
         <f>SUM(D4:D43)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>ממוצע פרמיה</t>
         </is>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="15">
         <f>AVERAGE(D4:D43)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>מזהה לקוח חסר</t>
         </is>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="15">
         <f>COUNTBLANK(F4:F43)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>כמות P-CAR</t>
         </is>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="15">
         <f>COUNTIF(C4:C43,"P-CAR")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>02</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>סה"כ פרמיה ל-P-HEALTH</t>
         </is>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="15">
         <f>SUMIF(C4:C43,"P-HEALTH",D4:D43)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>שם סוכן נקי</t>
         </is>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="15">
         <f>PROPER(TRIM(B4))</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>03</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t>כפילות</t>
         </is>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="15">
         <f>IF(COUNTIF($A$4:$A$43,A4)&gt;1,"כפול","ייחודי")</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>שם מוצר לפי קוד</t>
         </is>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="15">
         <f>IFERROR(VLOOKUP(B4,$H$5:$I$9,2,FALSE),"קוד לא קיים")</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>04</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>שם סוכן לפי קוד</t>
         </is>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="15">
         <f>IFERROR(INDEX($L$5:$L$9,MATCH(D4,$K$5:$K$9,0)),"קוד לא קיים")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>05</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>PivotTable</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>Insert &gt; PivotTable, Rows=שם סוכן, Values=Sum(פרמיה), Columns=סוג מוצר</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>פרמיה שלילית</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>New Rule &gt; Formula: =$D4&lt;0</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>תאריך עתידי</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>New Rule &gt; Formula: =$E4&gt;TODAY()</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>06</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>פוליסה כפולה</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>New Rule &gt; Formula: =COUNTIF($A$4:$A$43,$A4)&gt;1</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>שדה חובה</t>
         </is>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="15">
         <f>IF(F4="","חסר","תקין")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>כפילות</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="15">
         <f>IF(COUNTIF($A$4:$A$43,A4)&gt;1,"כפול","ייחודי")</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>07</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>החלטה סופית</t>
         </is>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="15">
         <f>IF(OR(G4="חסר",H4="כפול",D4&lt;0,E4&gt;TODAY()),"נדחה","קביל")</f>
         <v/>
       </c>
@@ -960,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1123,10 +1131,46 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>תרגול נוסף: Data Validation (רשימה נפתחת)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>דוגמה עובדת — לחצו על התא הבא לרשימה נפתחת:</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>ביטוח רכב</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>המשימה שלך: בתא B16 הוסיפו בעצמכם רשימה נפתחת דרך Data → Data Validation → Allow: List, עם הערכים: קביל,נדחה,בבדיקה — בדיוק כמו שדה 'סטטוס' שהיה נחוץ בתהליך קבילות נתונים אמיתי.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="11" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
+    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A12:E12"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B13" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ערך לא תקין" error="יש לבחור ערך מהרשימה בלבד" type="list">
+      <formula1>"ביטוח רכב,ביטוח דירה,ביטוח חיים,ביטוח בריאות,ביטוח נסיעות"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1203,10 +1247,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="12" t="n">
         <v>3414.51</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="13" t="n">
         <v>45177</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -1231,10 +1275,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="12" t="n">
         <v>3393.18</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="13" t="n">
         <v>45619</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -1259,10 +1303,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="12" t="n">
         <v>2780.07</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="13" t="n">
         <v>44959</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -1287,10 +1331,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="12" t="n">
         <v>1218.28</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="13" t="n">
         <v>45444</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -1315,10 +1359,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="12" t="n">
         <v>2657.23</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="13" t="n">
         <v>45660</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -1343,10 +1387,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="12" t="n">
         <v>1225.85</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="13" t="n">
         <v>45530</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -1371,10 +1415,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="12" t="n">
         <v>3486.99</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -1399,10 +1443,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="12" t="n">
         <v>1467.06</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="13" t="n">
         <v>45147</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -1427,10 +1471,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="12" t="n">
         <v>689.53</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="13" t="n">
         <v>45026</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -1455,10 +1499,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="12" t="n">
         <v>2835.65</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="13" t="n">
         <v>45753</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -1483,10 +1527,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="12" t="n">
         <v>2229.58</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="13" t="n">
         <v>45054</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -1511,10 +1555,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="12" t="n">
         <v>2618.57</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>45776</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -1539,10 +1583,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="12" t="n">
         <v>-150</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="13" t="n">
         <v>45648</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -1567,10 +1611,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="12" t="n">
         <v>3077.31</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>45718</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -1595,10 +1639,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="12" t="n">
         <v>3892.33</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="13" t="n">
         <v>45814</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -1623,10 +1667,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="12" t="n">
         <v>1467.49</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="13" t="n">
         <v>45577</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -1651,10 +1695,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="12" t="n">
         <v>1854.76</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="13" t="n">
         <v>45141</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -1679,10 +1723,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="12" t="n">
         <v>4233.95</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="13" t="n">
         <v>45590</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -1707,10 +1751,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="12" t="n">
         <v>2966.91</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="13" t="n">
         <v>45473</v>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1731,10 +1775,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="12" t="n">
         <v>2241.49</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="13" t="n">
         <v>45203</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -1759,10 +1803,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="12" t="n">
         <v>3175.38</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="13" t="n">
         <v>45790</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -1787,10 +1831,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>3751.57</v>
       </c>
-      <c r="E25" s="10" t="n">
+      <c r="E25" s="13" t="n">
         <v>45751</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -1815,10 +1859,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D26" s="12" t="n">
         <v>1424.51</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="13" t="n">
         <v>45143</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -1843,10 +1887,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" s="12" t="n">
         <v>1621.65</v>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="13" t="n">
         <v>45598</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -1871,10 +1915,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n">
+      <c r="D28" s="12" t="n">
         <v>4015.67</v>
       </c>
-      <c r="E28" s="10" t="n">
+      <c r="E28" s="13" t="n">
         <v>45585</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -1899,10 +1943,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D29" s="12" t="n">
         <v>1412.5</v>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="13" t="n">
         <v>45179</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -1927,10 +1971,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D30" s="9" t="n">
+      <c r="D30" s="12" t="n">
         <v>1403.51</v>
       </c>
-      <c r="E30" s="10" t="n">
+      <c r="E30" s="13" t="n">
         <v>45525</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -1955,10 +1999,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D31" s="12" t="n">
         <v>1977.48</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="13" t="n">
         <v>45151</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -1983,10 +2027,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D32" s="12" t="n">
         <v>2372.77</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="13" t="n">
         <v>45700</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -2011,10 +2055,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D33" s="12" t="n">
         <v>941.9299999999999</v>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -2039,10 +2083,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D34" s="9" t="n">
+      <c r="D34" s="12" t="n">
         <v>566.8200000000001</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="13" t="n">
         <v>46447</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -2067,10 +2111,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D35" s="9" t="n">
+      <c r="D35" s="12" t="n">
         <v>2522.28</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="13" t="n">
         <v>45493</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -2095,10 +2139,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D36" s="9" t="n">
+      <c r="D36" s="12" t="n">
         <v>3327.03</v>
       </c>
-      <c r="E36" s="10" t="n">
+      <c r="E36" s="13" t="n">
         <v>45625</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -2123,10 +2167,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" s="12" t="n">
         <v>3528.11</v>
       </c>
-      <c r="E37" s="10" t="n">
+      <c r="E37" s="13" t="n">
         <v>45275</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -2151,10 +2195,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D38" s="9" t="n">
+      <c r="D38" s="12" t="n">
         <v>2126.01</v>
       </c>
-      <c r="E38" s="10" t="n">
+      <c r="E38" s="13" t="n">
         <v>45391</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -2179,10 +2223,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D39" s="9" t="n">
+      <c r="D39" s="12" t="n">
         <v>3978.58</v>
       </c>
-      <c r="E39" s="10" t="n">
+      <c r="E39" s="13" t="n">
         <v>45196</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -2207,10 +2251,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="12" t="n">
         <v>2432.26</v>
       </c>
-      <c r="E40" s="10" t="n">
+      <c r="E40" s="13" t="n">
         <v>45035</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -2235,10 +2279,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="12" t="n">
         <v>2432.18</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="13" t="n">
         <v>45130</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -2263,10 +2307,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D42" s="9" t="n">
+      <c r="D42" s="12" t="n">
         <v>3502.55</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="13" t="n">
         <v>45479</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -2291,10 +2335,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n">
+      <c r="D43" s="12" t="n">
         <v>2815.57</v>
       </c>
-      <c r="E43" s="10" t="n">
+      <c r="E43" s="13" t="n">
         <v>45427</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -2316,7 +2360,7 @@
           <t>סה"כ פרמיה (SUM):</t>
         </is>
       </c>
-      <c r="B46" s="11">
+      <c r="B46" s="10">
         <f>SUM(D4:D43)</f>
         <v/>
       </c>
@@ -2327,7 +2371,7 @@
           <t>ממוצע פרמיה (AVERAGE):</t>
         </is>
       </c>
-      <c r="B47" s="11" t="n"/>
+      <c r="B47" s="10" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -2335,7 +2379,7 @@
           <t>כמה רשומות עם מזהה לקוח חסר (COUNTBLANK על עמודה F):</t>
         </is>
       </c>
-      <c r="B48" s="11" t="n"/>
+      <c r="B48" s="10" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
@@ -2343,7 +2387,7 @@
           <t>כמה פוליסות מסוג P-CAR (COUNTIF על עמודה C):</t>
         </is>
       </c>
-      <c r="B49" s="11" t="n"/>
+      <c r="B49" s="10" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -2351,7 +2395,7 @@
           <t>סה"כ פרמיה רק עבור P-HEALTH (SUMIF):</t>
         </is>
       </c>
-      <c r="B50" s="11" t="n"/>
+      <c r="B50" s="10" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2433,7 +2477,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="12" t="n">
         <v>3414.51</v>
       </c>
       <c r="E4" t="inlineStr"/>
@@ -2455,7 +2499,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="12" t="n">
         <v>3393.18</v>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -2477,7 +2521,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="12" t="n">
         <v>2780.07</v>
       </c>
       <c r="E6" t="inlineStr"/>
@@ -2499,7 +2543,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="12" t="n">
         <v>1218.28</v>
       </c>
       <c r="E7" t="inlineStr"/>
@@ -2521,7 +2565,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="12" t="n">
         <v>2657.23</v>
       </c>
       <c r="E8" t="inlineStr"/>
@@ -2543,7 +2587,7 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="12" t="n">
         <v>1225.85</v>
       </c>
       <c r="E9" t="inlineStr"/>
@@ -2565,7 +2609,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="12" t="n">
         <v>3486.99</v>
       </c>
       <c r="E10" t="inlineStr"/>
@@ -2587,7 +2631,7 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="12" t="n">
         <v>1467.06</v>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -2609,7 +2653,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="12" t="n">
         <v>689.53</v>
       </c>
       <c r="E12" t="inlineStr"/>
@@ -2631,7 +2675,7 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="12" t="n">
         <v>2835.65</v>
       </c>
       <c r="E13" t="inlineStr"/>
@@ -2653,7 +2697,7 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="12" t="n">
         <v>2229.58</v>
       </c>
       <c r="E14" t="inlineStr"/>
@@ -2675,7 +2719,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="12" t="n">
         <v>2618.57</v>
       </c>
       <c r="E15" t="inlineStr"/>
@@ -2697,7 +2741,7 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="12" t="n">
         <v>-150</v>
       </c>
       <c r="E16" t="inlineStr"/>
@@ -2719,7 +2763,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="12" t="n">
         <v>3077.31</v>
       </c>
       <c r="E17" t="inlineStr"/>
@@ -2741,7 +2785,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="12" t="n">
         <v>3892.33</v>
       </c>
       <c r="E18" t="inlineStr"/>
@@ -2763,7 +2807,7 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="12" t="n">
         <v>1467.49</v>
       </c>
       <c r="E19" t="inlineStr"/>
@@ -2785,7 +2829,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="12" t="n">
         <v>1854.76</v>
       </c>
       <c r="E20" t="inlineStr"/>
@@ -2807,7 +2851,7 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="12" t="n">
         <v>4233.95</v>
       </c>
       <c r="E21" t="inlineStr"/>
@@ -2829,7 +2873,7 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="12" t="n">
         <v>2966.91</v>
       </c>
       <c r="E22" t="inlineStr"/>
@@ -2851,7 +2895,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="12" t="n">
         <v>2241.49</v>
       </c>
       <c r="E23" t="inlineStr"/>
@@ -2873,7 +2917,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="12" t="n">
         <v>3175.38</v>
       </c>
       <c r="E24" t="inlineStr"/>
@@ -2895,7 +2939,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>3751.57</v>
       </c>
       <c r="E25" t="inlineStr"/>
@@ -2917,7 +2961,7 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D26" s="12" t="n">
         <v>1424.51</v>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -2939,7 +2983,7 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" s="12" t="n">
         <v>1621.65</v>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -2961,7 +3005,7 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n">
+      <c r="D28" s="12" t="n">
         <v>4015.67</v>
       </c>
       <c r="E28" t="inlineStr"/>
@@ -2983,7 +3027,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D29" s="12" t="n">
         <v>1412.5</v>
       </c>
       <c r="E29" t="inlineStr"/>
@@ -3005,7 +3049,7 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D30" s="9" t="n">
+      <c r="D30" s="12" t="n">
         <v>1403.51</v>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -3027,7 +3071,7 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D31" s="12" t="n">
         <v>1977.48</v>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -3049,7 +3093,7 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D32" s="12" t="n">
         <v>2372.77</v>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -3071,7 +3115,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D33" s="12" t="n">
         <v>941.9299999999999</v>
       </c>
       <c r="E33" t="inlineStr"/>
@@ -3093,7 +3137,7 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D34" s="9" t="n">
+      <c r="D34" s="12" t="n">
         <v>566.8200000000001</v>
       </c>
       <c r="E34" t="inlineStr"/>
@@ -3115,7 +3159,7 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D35" s="9" t="n">
+      <c r="D35" s="12" t="n">
         <v>2522.28</v>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -3137,7 +3181,7 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D36" s="9" t="n">
+      <c r="D36" s="12" t="n">
         <v>3327.03</v>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -3159,7 +3203,7 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" s="12" t="n">
         <v>3528.11</v>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -3181,7 +3225,7 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D38" s="9" t="n">
+      <c r="D38" s="12" t="n">
         <v>2126.01</v>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -3203,7 +3247,7 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D39" s="9" t="n">
+      <c r="D39" s="12" t="n">
         <v>3978.58</v>
       </c>
       <c r="E39" t="inlineStr"/>
@@ -3225,7 +3269,7 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="12" t="n">
         <v>2432.26</v>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -3247,7 +3291,7 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="12" t="n">
         <v>2432.18</v>
       </c>
       <c r="E41" t="inlineStr"/>
@@ -3269,7 +3313,7 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D42" s="9" t="n">
+      <c r="D42" s="12" t="n">
         <v>3502.55</v>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -3291,7 +3335,7 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n">
+      <c r="D43" s="12" t="n">
         <v>2815.57</v>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -4371,10 +4415,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="12" t="n">
         <v>3414.51</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="13" t="n">
         <v>45177</v>
       </c>
       <c r="F4">
@@ -4398,10 +4442,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="12" t="n">
         <v>3393.18</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="13" t="n">
         <v>45619</v>
       </c>
       <c r="F5">
@@ -4425,10 +4469,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="12" t="n">
         <v>2780.07</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="13" t="n">
         <v>44959</v>
       </c>
       <c r="F6">
@@ -4452,10 +4496,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="12" t="n">
         <v>1218.28</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="13" t="n">
         <v>45444</v>
       </c>
       <c r="F7">
@@ -4479,10 +4523,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="12" t="n">
         <v>2657.23</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="13" t="n">
         <v>45660</v>
       </c>
       <c r="F8">
@@ -4506,10 +4550,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="12" t="n">
         <v>1225.85</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="13" t="n">
         <v>45530</v>
       </c>
       <c r="F9">
@@ -4533,10 +4577,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="12" t="n">
         <v>3486.99</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F10">
@@ -4560,10 +4604,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="12" t="n">
         <v>1467.06</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="13" t="n">
         <v>45147</v>
       </c>
       <c r="F11">
@@ -4587,10 +4631,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="12" t="n">
         <v>689.53</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="13" t="n">
         <v>45026</v>
       </c>
       <c r="F12">
@@ -4614,10 +4658,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="12" t="n">
         <v>2835.65</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="13" t="n">
         <v>45753</v>
       </c>
       <c r="F13">
@@ -4641,10 +4685,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="12" t="n">
         <v>2229.58</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="13" t="n">
         <v>45054</v>
       </c>
       <c r="F14">
@@ -4668,10 +4712,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="12" t="n">
         <v>2618.57</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>45776</v>
       </c>
       <c r="F15">
@@ -4695,10 +4739,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="12" t="n">
         <v>-150</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="13" t="n">
         <v>45648</v>
       </c>
       <c r="F16">
@@ -4722,10 +4766,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="12" t="n">
         <v>3077.31</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>45718</v>
       </c>
       <c r="F17">
@@ -4749,10 +4793,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="12" t="n">
         <v>3892.33</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="13" t="n">
         <v>45814</v>
       </c>
       <c r="F18">
@@ -4776,10 +4820,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="12" t="n">
         <v>1467.49</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="13" t="n">
         <v>45577</v>
       </c>
       <c r="F19">
@@ -4803,10 +4847,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="12" t="n">
         <v>1854.76</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="13" t="n">
         <v>45141</v>
       </c>
       <c r="F20">
@@ -4830,10 +4874,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="12" t="n">
         <v>4233.95</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="13" t="n">
         <v>45590</v>
       </c>
       <c r="F21">
@@ -4857,10 +4901,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="12" t="n">
         <v>2966.91</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="13" t="n">
         <v>45473</v>
       </c>
       <c r="F22">
@@ -4884,10 +4928,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="12" t="n">
         <v>2241.49</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="13" t="n">
         <v>45203</v>
       </c>
       <c r="F23">
@@ -4911,10 +4955,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="12" t="n">
         <v>3175.38</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="13" t="n">
         <v>45790</v>
       </c>
       <c r="F24">
@@ -4938,10 +4982,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>3751.57</v>
       </c>
-      <c r="E25" s="10" t="n">
+      <c r="E25" s="13" t="n">
         <v>45751</v>
       </c>
       <c r="F25">
@@ -4965,10 +5009,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D26" s="12" t="n">
         <v>1424.51</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="13" t="n">
         <v>45143</v>
       </c>
       <c r="F26">
@@ -4992,10 +5036,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" s="12" t="n">
         <v>1621.65</v>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="13" t="n">
         <v>45598</v>
       </c>
       <c r="F27">
@@ -5019,10 +5063,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n">
+      <c r="D28" s="12" t="n">
         <v>4015.67</v>
       </c>
-      <c r="E28" s="10" t="n">
+      <c r="E28" s="13" t="n">
         <v>45585</v>
       </c>
       <c r="F28">
@@ -5046,10 +5090,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D29" s="12" t="n">
         <v>1412.5</v>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="13" t="n">
         <v>45179</v>
       </c>
       <c r="F29">
@@ -5073,10 +5117,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D30" s="9" t="n">
+      <c r="D30" s="12" t="n">
         <v>1403.51</v>
       </c>
-      <c r="E30" s="10" t="n">
+      <c r="E30" s="13" t="n">
         <v>45525</v>
       </c>
       <c r="F30">
@@ -5100,10 +5144,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D31" s="12" t="n">
         <v>1977.48</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="13" t="n">
         <v>45151</v>
       </c>
       <c r="F31">
@@ -5127,10 +5171,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D32" s="12" t="n">
         <v>2372.77</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="13" t="n">
         <v>45700</v>
       </c>
       <c r="F32">
@@ -5154,10 +5198,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D33" s="12" t="n">
         <v>941.9299999999999</v>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F33">
@@ -5181,10 +5225,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D34" s="9" t="n">
+      <c r="D34" s="12" t="n">
         <v>566.8200000000001</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="13" t="n">
         <v>46447</v>
       </c>
       <c r="F34">
@@ -5208,10 +5252,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D35" s="9" t="n">
+      <c r="D35" s="12" t="n">
         <v>2522.28</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="13" t="n">
         <v>45493</v>
       </c>
       <c r="F35">
@@ -5235,10 +5279,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D36" s="9" t="n">
+      <c r="D36" s="12" t="n">
         <v>3327.03</v>
       </c>
-      <c r="E36" s="10" t="n">
+      <c r="E36" s="13" t="n">
         <v>45625</v>
       </c>
       <c r="F36">
@@ -5262,10 +5306,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" s="12" t="n">
         <v>3528.11</v>
       </c>
-      <c r="E37" s="10" t="n">
+      <c r="E37" s="13" t="n">
         <v>45275</v>
       </c>
       <c r="F37">
@@ -5289,10 +5333,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D38" s="9" t="n">
+      <c r="D38" s="12" t="n">
         <v>2126.01</v>
       </c>
-      <c r="E38" s="10" t="n">
+      <c r="E38" s="13" t="n">
         <v>45391</v>
       </c>
       <c r="F38">
@@ -5316,10 +5360,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D39" s="9" t="n">
+      <c r="D39" s="12" t="n">
         <v>3978.58</v>
       </c>
-      <c r="E39" s="10" t="n">
+      <c r="E39" s="13" t="n">
         <v>45196</v>
       </c>
       <c r="F39">
@@ -5343,10 +5387,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="12" t="n">
         <v>2432.26</v>
       </c>
-      <c r="E40" s="10" t="n">
+      <c r="E40" s="13" t="n">
         <v>45035</v>
       </c>
       <c r="F40">
@@ -5370,10 +5414,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="12" t="n">
         <v>2432.18</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="13" t="n">
         <v>45130</v>
       </c>
       <c r="F41">
@@ -5397,10 +5441,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D42" s="9" t="n">
+      <c r="D42" s="12" t="n">
         <v>3502.55</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="13" t="n">
         <v>45479</v>
       </c>
       <c r="F42">
@@ -5424,10 +5468,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n">
+      <c r="D43" s="12" t="n">
         <v>2815.57</v>
       </c>
-      <c r="E43" s="10" t="n">
+      <c r="E43" s="13" t="n">
         <v>45427</v>
       </c>
       <c r="F43">
@@ -5547,10 +5591,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="12" t="n">
         <v>3414.51</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="13" t="n">
         <v>45177</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -5575,10 +5619,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="12" t="n">
         <v>3393.18</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="13" t="n">
         <v>45619</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -5603,10 +5647,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="12" t="n">
         <v>2780.07</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="13" t="n">
         <v>44959</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -5631,10 +5675,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="12" t="n">
         <v>1218.28</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="13" t="n">
         <v>45444</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -5659,10 +5703,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="12" t="n">
         <v>2657.23</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="13" t="n">
         <v>45660</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -5687,10 +5731,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="12" t="n">
         <v>1225.85</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="13" t="n">
         <v>45530</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -5715,10 +5759,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="12" t="n">
         <v>3486.99</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -5743,10 +5787,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="12" t="n">
         <v>1467.06</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="13" t="n">
         <v>45147</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -5771,10 +5815,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="12" t="n">
         <v>689.53</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="13" t="n">
         <v>45026</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -5799,10 +5843,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="12" t="n">
         <v>2835.65</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="13" t="n">
         <v>45753</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -5827,10 +5871,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="12" t="n">
         <v>2229.58</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="13" t="n">
         <v>45054</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -5855,10 +5899,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="12" t="n">
         <v>2618.57</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>45776</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -5883,10 +5927,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="12" t="n">
         <v>-150</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="13" t="n">
         <v>45648</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -5911,10 +5955,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="12" t="n">
         <v>3077.31</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>45718</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -5939,10 +5983,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="12" t="n">
         <v>3892.33</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="13" t="n">
         <v>45814</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -5967,10 +6011,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="12" t="n">
         <v>1467.49</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="13" t="n">
         <v>45577</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -5995,10 +6039,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="12" t="n">
         <v>1854.76</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="13" t="n">
         <v>45141</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -6023,10 +6067,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="12" t="n">
         <v>4233.95</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="13" t="n">
         <v>45590</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -6051,10 +6095,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="12" t="n">
         <v>2966.91</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="13" t="n">
         <v>45473</v>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -6075,10 +6119,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="12" t="n">
         <v>2241.49</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="13" t="n">
         <v>45203</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -6103,10 +6147,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="12" t="n">
         <v>3175.38</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="13" t="n">
         <v>45790</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -6131,10 +6175,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>3751.57</v>
       </c>
-      <c r="E25" s="10" t="n">
+      <c r="E25" s="13" t="n">
         <v>45751</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -6159,10 +6203,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D26" s="12" t="n">
         <v>1424.51</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="13" t="n">
         <v>45143</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -6187,10 +6231,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" s="12" t="n">
         <v>1621.65</v>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="13" t="n">
         <v>45598</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -6215,10 +6259,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n">
+      <c r="D28" s="12" t="n">
         <v>4015.67</v>
       </c>
-      <c r="E28" s="10" t="n">
+      <c r="E28" s="13" t="n">
         <v>45585</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -6243,10 +6287,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D29" s="12" t="n">
         <v>1412.5</v>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="13" t="n">
         <v>45179</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -6271,10 +6315,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D30" s="9" t="n">
+      <c r="D30" s="12" t="n">
         <v>1403.51</v>
       </c>
-      <c r="E30" s="10" t="n">
+      <c r="E30" s="13" t="n">
         <v>45525</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -6299,10 +6343,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D31" s="12" t="n">
         <v>1977.48</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="13" t="n">
         <v>45151</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -6327,10 +6371,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D32" s="12" t="n">
         <v>2372.77</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="13" t="n">
         <v>45700</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -6355,10 +6399,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D33" s="12" t="n">
         <v>941.9299999999999</v>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -6383,10 +6427,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D34" s="9" t="n">
+      <c r="D34" s="12" t="n">
         <v>566.8200000000001</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="13" t="n">
         <v>46447</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -6411,10 +6455,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D35" s="9" t="n">
+      <c r="D35" s="12" t="n">
         <v>2522.28</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="13" t="n">
         <v>45493</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -6439,10 +6483,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D36" s="9" t="n">
+      <c r="D36" s="12" t="n">
         <v>3327.03</v>
       </c>
-      <c r="E36" s="10" t="n">
+      <c r="E36" s="13" t="n">
         <v>45625</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -6467,10 +6511,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" s="12" t="n">
         <v>3528.11</v>
       </c>
-      <c r="E37" s="10" t="n">
+      <c r="E37" s="13" t="n">
         <v>45275</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -6495,10 +6539,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D38" s="9" t="n">
+      <c r="D38" s="12" t="n">
         <v>2126.01</v>
       </c>
-      <c r="E38" s="10" t="n">
+      <c r="E38" s="13" t="n">
         <v>45391</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -6523,10 +6567,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D39" s="9" t="n">
+      <c r="D39" s="12" t="n">
         <v>3978.58</v>
       </c>
-      <c r="E39" s="10" t="n">
+      <c r="E39" s="13" t="n">
         <v>45196</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -6551,10 +6595,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="12" t="n">
         <v>2432.26</v>
       </c>
-      <c r="E40" s="10" t="n">
+      <c r="E40" s="13" t="n">
         <v>45035</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -6579,10 +6623,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="12" t="n">
         <v>2432.18</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="13" t="n">
         <v>45130</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -6607,10 +6651,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D42" s="9" t="n">
+      <c r="D42" s="12" t="n">
         <v>3502.55</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="13" t="n">
         <v>45479</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -6635,10 +6679,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n">
+      <c r="D43" s="12" t="n">
         <v>2815.57</v>
       </c>
-      <c r="E43" s="10" t="n">
+      <c r="E43" s="13" t="n">
         <v>45427</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -6785,10 +6829,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D4" s="9" t="n">
+      <c r="D4" s="12" t="n">
         <v>3414.51</v>
       </c>
-      <c r="E4" s="10" t="n">
+      <c r="E4" s="13" t="n">
         <v>45177</v>
       </c>
       <c r="F4" t="inlineStr">
@@ -6816,10 +6860,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="12" t="n">
         <v>3393.18</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E5" s="13" t="n">
         <v>45619</v>
       </c>
       <c r="F5" t="inlineStr">
@@ -6847,10 +6891,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="12" t="n">
         <v>2780.07</v>
       </c>
-      <c r="E6" s="10" t="n">
+      <c r="E6" s="13" t="n">
         <v>44959</v>
       </c>
       <c r="F6" t="inlineStr">
@@ -6878,10 +6922,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="12" t="n">
         <v>1218.28</v>
       </c>
-      <c r="E7" s="10" t="n">
+      <c r="E7" s="13" t="n">
         <v>45444</v>
       </c>
       <c r="F7" t="inlineStr">
@@ -6909,10 +6953,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="12" t="n">
         <v>2657.23</v>
       </c>
-      <c r="E8" s="10" t="n">
+      <c r="E8" s="13" t="n">
         <v>45660</v>
       </c>
       <c r="F8" t="inlineStr">
@@ -6940,10 +6984,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n">
+      <c r="D9" s="12" t="n">
         <v>1225.85</v>
       </c>
-      <c r="E9" s="10" t="n">
+      <c r="E9" s="13" t="n">
         <v>45530</v>
       </c>
       <c r="F9" t="inlineStr">
@@ -6971,10 +7015,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="12" t="n">
         <v>3486.99</v>
       </c>
-      <c r="E10" s="10" t="n">
+      <c r="E10" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F10" t="inlineStr">
@@ -7002,10 +7046,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="12" t="n">
         <v>1467.06</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E11" s="13" t="n">
         <v>45147</v>
       </c>
       <c r="F11" t="inlineStr">
@@ -7033,10 +7077,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="12" t="n">
         <v>689.53</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="13" t="n">
         <v>45026</v>
       </c>
       <c r="F12" t="inlineStr">
@@ -7064,10 +7108,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="12" t="n">
         <v>2835.65</v>
       </c>
-      <c r="E13" s="10" t="n">
+      <c r="E13" s="13" t="n">
         <v>45753</v>
       </c>
       <c r="F13" t="inlineStr">
@@ -7095,10 +7139,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="12" t="n">
         <v>2229.58</v>
       </c>
-      <c r="E14" s="10" t="n">
+      <c r="E14" s="13" t="n">
         <v>45054</v>
       </c>
       <c r="F14" t="inlineStr">
@@ -7126,10 +7170,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="12" t="n">
         <v>2618.57</v>
       </c>
-      <c r="E15" s="10" t="n">
+      <c r="E15" s="13" t="n">
         <v>45776</v>
       </c>
       <c r="F15" t="inlineStr">
@@ -7157,10 +7201,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="12" t="n">
         <v>-150</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E16" s="13" t="n">
         <v>45648</v>
       </c>
       <c r="F16" t="inlineStr">
@@ -7188,10 +7232,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="12" t="n">
         <v>3077.31</v>
       </c>
-      <c r="E17" s="10" t="n">
+      <c r="E17" s="13" t="n">
         <v>45718</v>
       </c>
       <c r="F17" t="inlineStr">
@@ -7219,10 +7263,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D18" s="9" t="n">
+      <c r="D18" s="12" t="n">
         <v>3892.33</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="13" t="n">
         <v>45814</v>
       </c>
       <c r="F18" t="inlineStr">
@@ -7250,10 +7294,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D19" s="9" t="n">
+      <c r="D19" s="12" t="n">
         <v>1467.49</v>
       </c>
-      <c r="E19" s="10" t="n">
+      <c r="E19" s="13" t="n">
         <v>45577</v>
       </c>
       <c r="F19" t="inlineStr">
@@ -7281,10 +7325,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="D20" s="12" t="n">
         <v>1854.76</v>
       </c>
-      <c r="E20" s="10" t="n">
+      <c r="E20" s="13" t="n">
         <v>45141</v>
       </c>
       <c r="F20" t="inlineStr">
@@ -7312,10 +7356,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n">
+      <c r="D21" s="12" t="n">
         <v>4233.95</v>
       </c>
-      <c r="E21" s="10" t="n">
+      <c r="E21" s="13" t="n">
         <v>45590</v>
       </c>
       <c r="F21" t="inlineStr">
@@ -7343,10 +7387,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D22" s="9" t="n">
+      <c r="D22" s="12" t="n">
         <v>2966.91</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="13" t="n">
         <v>45473</v>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -7370,10 +7414,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="12" t="n">
         <v>2241.49</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E23" s="13" t="n">
         <v>45203</v>
       </c>
       <c r="F23" t="inlineStr">
@@ -7401,10 +7445,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D24" s="9" t="n">
+      <c r="D24" s="12" t="n">
         <v>3175.38</v>
       </c>
-      <c r="E24" s="10" t="n">
+      <c r="E24" s="13" t="n">
         <v>45790</v>
       </c>
       <c r="F24" t="inlineStr">
@@ -7432,10 +7476,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="D25" s="12" t="n">
         <v>3751.57</v>
       </c>
-      <c r="E25" s="10" t="n">
+      <c r="E25" s="13" t="n">
         <v>45751</v>
       </c>
       <c r="F25" t="inlineStr">
@@ -7463,10 +7507,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D26" s="9" t="n">
+      <c r="D26" s="12" t="n">
         <v>1424.51</v>
       </c>
-      <c r="E26" s="10" t="n">
+      <c r="E26" s="13" t="n">
         <v>45143</v>
       </c>
       <c r="F26" t="inlineStr">
@@ -7494,10 +7538,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="D27" s="12" t="n">
         <v>1621.65</v>
       </c>
-      <c r="E27" s="10" t="n">
+      <c r="E27" s="13" t="n">
         <v>45598</v>
       </c>
       <c r="F27" t="inlineStr">
@@ -7525,10 +7569,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n">
+      <c r="D28" s="12" t="n">
         <v>4015.67</v>
       </c>
-      <c r="E28" s="10" t="n">
+      <c r="E28" s="13" t="n">
         <v>45585</v>
       </c>
       <c r="F28" t="inlineStr">
@@ -7556,10 +7600,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="D29" s="12" t="n">
         <v>1412.5</v>
       </c>
-      <c r="E29" s="10" t="n">
+      <c r="E29" s="13" t="n">
         <v>45179</v>
       </c>
       <c r="F29" t="inlineStr">
@@ -7587,10 +7631,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D30" s="9" t="n">
+      <c r="D30" s="12" t="n">
         <v>1403.51</v>
       </c>
-      <c r="E30" s="10" t="n">
+      <c r="E30" s="13" t="n">
         <v>45525</v>
       </c>
       <c r="F30" t="inlineStr">
@@ -7618,10 +7662,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="D31" s="12" t="n">
         <v>1977.48</v>
       </c>
-      <c r="E31" s="10" t="n">
+      <c r="E31" s="13" t="n">
         <v>45151</v>
       </c>
       <c r="F31" t="inlineStr">
@@ -7649,10 +7693,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D32" s="9" t="n">
+      <c r="D32" s="12" t="n">
         <v>2372.77</v>
       </c>
-      <c r="E32" s="10" t="n">
+      <c r="E32" s="13" t="n">
         <v>45700</v>
       </c>
       <c r="F32" t="inlineStr">
@@ -7680,10 +7724,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D33" s="9" t="n">
+      <c r="D33" s="12" t="n">
         <v>941.9299999999999</v>
       </c>
-      <c r="E33" s="10" t="n">
+      <c r="E33" s="13" t="n">
         <v>45090</v>
       </c>
       <c r="F33" t="inlineStr">
@@ -7711,10 +7755,10 @@
           <t>P-TRAVEL</t>
         </is>
       </c>
-      <c r="D34" s="9" t="n">
+      <c r="D34" s="12" t="n">
         <v>566.8200000000001</v>
       </c>
-      <c r="E34" s="10" t="n">
+      <c r="E34" s="13" t="n">
         <v>46447</v>
       </c>
       <c r="F34" t="inlineStr">
@@ -7742,10 +7786,10 @@
           <t>P-HEALTH</t>
         </is>
       </c>
-      <c r="D35" s="9" t="n">
+      <c r="D35" s="12" t="n">
         <v>2522.28</v>
       </c>
-      <c r="E35" s="10" t="n">
+      <c r="E35" s="13" t="n">
         <v>45493</v>
       </c>
       <c r="F35" t="inlineStr">
@@ -7773,10 +7817,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D36" s="9" t="n">
+      <c r="D36" s="12" t="n">
         <v>3327.03</v>
       </c>
-      <c r="E36" s="10" t="n">
+      <c r="E36" s="13" t="n">
         <v>45625</v>
       </c>
       <c r="F36" t="inlineStr">
@@ -7804,10 +7848,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D37" s="9" t="n">
+      <c r="D37" s="12" t="n">
         <v>3528.11</v>
       </c>
-      <c r="E37" s="10" t="n">
+      <c r="E37" s="13" t="n">
         <v>45275</v>
       </c>
       <c r="F37" t="inlineStr">
@@ -7835,10 +7879,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D38" s="9" t="n">
+      <c r="D38" s="12" t="n">
         <v>2126.01</v>
       </c>
-      <c r="E38" s="10" t="n">
+      <c r="E38" s="13" t="n">
         <v>45391</v>
       </c>
       <c r="F38" t="inlineStr">
@@ -7866,10 +7910,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D39" s="9" t="n">
+      <c r="D39" s="12" t="n">
         <v>3978.58</v>
       </c>
-      <c r="E39" s="10" t="n">
+      <c r="E39" s="13" t="n">
         <v>45196</v>
       </c>
       <c r="F39" t="inlineStr">
@@ -7897,10 +7941,10 @@
           <t>P-HOME</t>
         </is>
       </c>
-      <c r="D40" s="9" t="n">
+      <c r="D40" s="12" t="n">
         <v>2432.26</v>
       </c>
-      <c r="E40" s="10" t="n">
+      <c r="E40" s="13" t="n">
         <v>45035</v>
       </c>
       <c r="F40" t="inlineStr">
@@ -7928,10 +7972,10 @@
           <t>P-PET</t>
         </is>
       </c>
-      <c r="D41" s="9" t="n">
+      <c r="D41" s="12" t="n">
         <v>2432.18</v>
       </c>
-      <c r="E41" s="10" t="n">
+      <c r="E41" s="13" t="n">
         <v>45130</v>
       </c>
       <c r="F41" t="inlineStr">
@@ -7959,10 +8003,10 @@
           <t>P-LIFE</t>
         </is>
       </c>
-      <c r="D42" s="9" t="n">
+      <c r="D42" s="12" t="n">
         <v>3502.55</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="13" t="n">
         <v>45479</v>
       </c>
       <c r="F42" t="inlineStr">
@@ -7990,10 +8034,10 @@
           <t>P-CAR</t>
         </is>
       </c>
-      <c r="D43" s="9" t="n">
+      <c r="D43" s="12" t="n">
         <v>2815.57</v>
       </c>
-      <c r="E43" s="10" t="n">
+      <c r="E43" s="13" t="n">
         <v>45427</v>
       </c>
       <c r="F43" t="inlineStr">
@@ -8078,7 +8122,7 @@
       <c r="A4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>שלבים:</t>
         </is>
@@ -8137,7 +8181,7 @@
       <c r="A13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>היתרון על פני נוסחאות: כל שלב נשמר ורשום ב-Applied Steps. אם מגיע קובץ חדש עם אותו מבנה, מספיק ללחוץ Data → Refresh All וכל תהליך הניקוי רץ מחדש אוטומטית — בלי לגרור נוסחאות מחדש.</t>
         </is>
@@ -8147,7 +8191,7 @@
       <c r="A15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>לחיזוק: נסו למזג (Merge Queries) את הנתונים הנקיים מול טבלת המוצרים בגיליון '04_VLOOKUP' (עמודות H:I) — זו הדרך של Power Query לעשות VLOOKUP, רק שקופה וניתנת לתיעוד.</t>
         </is>

</xml_diff>